<commit_message>
Atualiza planilhas de cenário e controles
</commit_message>
<xml_diff>
--- a/CENARIO ATUAL CARLOS FERNANDES E GISELLE.xlsx
+++ b/CENARIO ATUAL CARLOS FERNANDES E GISELLE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\MEDICOES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AABC45E-1C12-4BD7-979E-432465F8DBD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685F0C83-D4D1-451D-A4EC-C14B9A2ABB05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{137AA420-8DEA-448A-9601-757C9AEBEDC8}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{137AA420-8DEA-448A-9601-757C9AEBEDC8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="104">
   <si>
     <t>CONTRATADA</t>
   </si>
@@ -303,6 +303,51 @@
   </si>
   <si>
     <t>CENÁRIO ATUAL - GISELLE GONÇALVES DA FONSECA</t>
+  </si>
+  <si>
+    <t>Fiscal atuante</t>
+  </si>
+  <si>
+    <t>Fiscal Suplente</t>
+  </si>
+  <si>
+    <t>Giselle</t>
+  </si>
+  <si>
+    <t>Otavio</t>
+  </si>
+  <si>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>Oswaldo e Otavio</t>
+  </si>
+  <si>
+    <t>Rio da Flores</t>
+  </si>
+  <si>
+    <t>Otavio E Higor</t>
+  </si>
+  <si>
+    <t>Luciana E Otavio</t>
+  </si>
+  <si>
+    <t>Higor</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Luciana</t>
+  </si>
+  <si>
+    <t>Luciana e Oswaldo</t>
+  </si>
+  <si>
+    <t>Luciana E Oswaldo</t>
+  </si>
+  <si>
+    <t>Carlos Fernandes</t>
   </si>
 </sst>
 </file>
@@ -349,7 +394,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -362,8 +407,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <gradientFill degree="90">
+        <stop position="0">
+          <color theme="0"/>
+        </stop>
+        <stop position="1">
+          <color theme="0"/>
+        </stop>
+      </gradientFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -386,12 +441,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -407,108 +475,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDE205"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF962A2A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF97B2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF32586D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFABD1C9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF20C49C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF147B93"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB0EDC4"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <b/>
@@ -1013,7 +996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4D0DCF7-C013-4332-B7F3-2D555ED0B379}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr defaultRowHeight="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -1022,9 +1005,14 @@
     <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>88</v>
       </c>
@@ -1033,7 +1021,7 @@
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
     </row>
-    <row r="2" spans="1:5" s="3" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="3" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>86</v>
       </c>
@@ -1049,8 +1037,15 @@
       <c r="E2" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I2"/>
+      <c r="J2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+    </row>
+    <row r="3" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1066,8 +1061,21 @@
       <c r="E3" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I3" s="3"/>
+      <c r="J3" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="M3" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1083,8 +1091,23 @@
       <c r="E4" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1100,8 +1123,23 @@
       <c r="E5" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -1117,8 +1155,23 @@
       <c r="E6" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -1134,8 +1187,23 @@
       <c r="E7" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1151,8 +1219,23 @@
       <c r="E8" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
@@ -1168,8 +1251,23 @@
       <c r="E9" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
@@ -1186,7 +1284,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
@@ -1202,8 +1300,14 @@
       <c r="E11" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J11" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+    </row>
+    <row r="12" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
@@ -1219,8 +1323,20 @@
       <c r="E12" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J12" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -1236,8 +1352,23 @@
       <c r="E13" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1254,7 +1385,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -1271,7 +1402,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
@@ -1617,9 +1748,11 @@
       <c r="E39" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A20:E20"/>
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="J11:M11"/>
   </mergeCells>
   <conditionalFormatting sqref="E2">
     <cfRule type="containsText" dxfId="15" priority="9" operator="containsText" text="PRÉVIA">

</xml_diff>